<commit_message>
Faculty Subject Allocation: initial implementation and business rule improvements
</commit_message>
<xml_diff>
--- a/Faculty_Template.xlsx
+++ b/Faculty_Template.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="555" windowWidth="19815" windowHeight="7365"/>
+    <workbookView xWindow="510" yWindow="570" windowWidth="13095" windowHeight="5580"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="53">
   <si>
     <t>* Employee Code</t>
   </si>
@@ -41,6 +41,9 @@
     <t>Email</t>
   </si>
   <si>
+    <t>* PAN Card No</t>
+  </si>
+  <si>
     <t>Gender</t>
   </si>
   <si>
@@ -80,6 +83,9 @@
     <t>faculty@college.edu</t>
   </si>
   <si>
+    <t>ABCDE1234F</t>
+  </si>
+  <si>
     <t>Male</t>
   </si>
   <si>
@@ -147,13 +153,34 @@
   </si>
   <si>
     <t>Do not delete mandatory columns.</t>
+  </si>
+  <si>
+    <t>EMP002</t>
+  </si>
+  <si>
+    <t>Preti</t>
+  </si>
+  <si>
+    <t>Professor</t>
+  </si>
+  <si>
+    <t>peeti@gmail.com</t>
+  </si>
+  <si>
+    <t>MMMMM1234F</t>
+  </si>
+  <si>
+    <t>Female</t>
+  </si>
+  <si>
+    <t>Mechanical Engineering</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -166,7 +193,14 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -192,16 +226,19 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -215,9 +252,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImportTable" displayName="ImportTable" ref="A1:N5">
-  <autoFilter ref="A1:N5"/>
-  <tableColumns count="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImportTable" displayName="ImportTable" ref="A1:O3">
+  <autoFilter ref="A1:O3"/>
+  <tableColumns count="15">
     <tableColumn id="1" name="* Employee Code"/>
     <tableColumn id="2" name="* First Name"/>
     <tableColumn id="3" name="Middle Name"/>
@@ -226,12 +263,13 @@
     <tableColumn id="6" name="* Designation"/>
     <tableColumn id="7" name="Mobile"/>
     <tableColumn id="8" name="Email"/>
-    <tableColumn id="9" name="Gender"/>
-    <tableColumn id="10" name="Qualification"/>
-    <tableColumn id="11" name="Experience"/>
-    <tableColumn id="12" name="Joining Date"/>
-    <tableColumn id="13" name="Employment Type"/>
-    <tableColumn id="14" name="Specialization"/>
+    <tableColumn id="9" name="* PAN Card No"/>
+    <tableColumn id="10" name="Gender"/>
+    <tableColumn id="11" name="Qualification"/>
+    <tableColumn id="12" name="Experience"/>
+    <tableColumn id="13" name="Joining Date"/>
+    <tableColumn id="14" name="Employment Type"/>
+    <tableColumn id="15" name="Specialization"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -522,7 +560,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:O3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -532,15 +570,16 @@
     <col min="6" max="6" width="24" customWidth="1"/>
     <col min="7" max="7" width="15" customWidth="1"/>
     <col min="8" max="8" width="24" customWidth="1"/>
-    <col min="9" max="9" width="11" customWidth="1"/>
-    <col min="10" max="10" width="18" customWidth="1"/>
-    <col min="11" max="11" width="15" customWidth="1"/>
-    <col min="12" max="12" width="17" customWidth="1"/>
-    <col min="13" max="13" width="20" customWidth="1"/>
-    <col min="14" max="14" width="19" customWidth="1"/>
+    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="10" max="10" width="11" customWidth="1"/>
+    <col min="11" max="11" width="18" customWidth="1"/>
+    <col min="12" max="12" width="15" customWidth="1"/>
+    <col min="13" max="13" width="17" customWidth="1"/>
+    <col min="14" max="14" width="20" customWidth="1"/>
+    <col min="15" max="15" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -583,175 +622,90 @@
       <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M2" t="s">
+        <v>26</v>
+      </c>
+      <c r="N2" t="s">
+        <v>27</v>
+      </c>
+      <c r="O2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D3" t="s">
         <v>17</v>
       </c>
-      <c r="F2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G2" t="s">
-        <v>19</v>
-      </c>
-      <c r="H2" t="s">
-        <v>20</v>
-      </c>
-      <c r="I2" t="s">
-        <v>21</v>
-      </c>
-      <c r="J2" t="s">
-        <v>22</v>
-      </c>
-      <c r="K2" t="s">
-        <v>23</v>
-      </c>
-      <c r="L2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D3" t="s">
-        <v>16</v>
-      </c>
       <c r="E3" t="s">
-        <v>17</v>
+        <v>52</v>
       </c>
       <c r="F3" t="s">
-        <v>18</v>
-      </c>
-      <c r="G3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H3" t="s">
-        <v>20</v>
+        <v>48</v>
+      </c>
+      <c r="G3">
+        <v>7777777777</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>49</v>
       </c>
       <c r="I3" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="J3" t="s">
-        <v>22</v>
-      </c>
-      <c r="K3" t="s">
-        <v>23</v>
-      </c>
-      <c r="L3" t="s">
-        <v>24</v>
-      </c>
-      <c r="M3" t="s">
-        <v>25</v>
-      </c>
-      <c r="N3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" t="s">
-        <v>15</v>
-      </c>
-      <c r="D4" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G4" t="s">
-        <v>19</v>
-      </c>
-      <c r="H4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I4" t="s">
-        <v>21</v>
-      </c>
-      <c r="J4" t="s">
-        <v>22</v>
-      </c>
-      <c r="K4" t="s">
-        <v>23</v>
-      </c>
-      <c r="L4" t="s">
-        <v>24</v>
-      </c>
-      <c r="M4" t="s">
-        <v>25</v>
-      </c>
-      <c r="N4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" t="s">
-        <v>16</v>
-      </c>
-      <c r="E5" t="s">
-        <v>17</v>
-      </c>
-      <c r="F5" t="s">
-        <v>18</v>
-      </c>
-      <c r="G5" t="s">
-        <v>19</v>
-      </c>
-      <c r="H5" t="s">
-        <v>20</v>
-      </c>
-      <c r="I5" t="s">
-        <v>21</v>
-      </c>
-      <c r="J5" t="s">
-        <v>22</v>
-      </c>
-      <c r="K5" t="s">
-        <v>23</v>
-      </c>
-      <c r="L5" t="s">
-        <v>24</v>
-      </c>
-      <c r="M5" t="s">
-        <v>25</v>
-      </c>
-      <c r="N5" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="H3" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -767,42 +721,42 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -810,7 +764,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -818,31 +772,31 @@
         <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B8" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B10" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactor Batch Management UI layout skeleton
</commit_message>
<xml_diff>
--- a/Faculty_Template.xlsx
+++ b/Faculty_Template.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="60">
   <si>
     <t>* Employee Code</t>
   </si>
@@ -174,6 +174,27 @@
   </si>
   <si>
     <t>Mechanical Engineering</t>
+  </si>
+  <si>
+    <t>EMP004</t>
+  </si>
+  <si>
+    <t>afdsaf</t>
+  </si>
+  <si>
+    <t>dsafs</t>
+  </si>
+  <si>
+    <t>sadfsdf</t>
+  </si>
+  <si>
+    <t>Electrical Engineering</t>
+  </si>
+  <si>
+    <t>asddsa@gmail.com</t>
+  </si>
+  <si>
+    <t>fffff1111S</t>
   </si>
 </sst>
 </file>
@@ -252,8 +273,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImportTable" displayName="ImportTable" ref="A1:O3">
-  <autoFilter ref="A1:O3"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImportTable" displayName="ImportTable" ref="A1:O4">
+  <autoFilter ref="A1:O4"/>
   <tableColumns count="15">
     <tableColumn id="1" name="* Employee Code"/>
     <tableColumn id="2" name="* First Name"/>
@@ -560,7 +581,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O3"/>
+  <dimension ref="A1:O4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -699,13 +720,43 @@
         <v>51</v>
       </c>
     </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D4" t="s">
+        <v>56</v>
+      </c>
+      <c r="E4" t="s">
+        <v>57</v>
+      </c>
+      <c r="F4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G4">
+        <v>1212121212</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="I4" t="s">
+        <v>59</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="H3" r:id="rId1"/>
+    <hyperlink ref="H4" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Faculty Subject Allocation: dynamic loading, row selection, CRUD fixes, UI improvements
</commit_message>
<xml_diff>
--- a/Faculty_Template.xlsx
+++ b/Faculty_Template.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="96">
   <si>
     <t>* Employee Code</t>
   </si>
@@ -62,48 +62,12 @@
     <t>Specialization</t>
   </si>
   <si>
-    <t>EMP001</t>
-  </si>
-  <si>
-    <t>Pramod</t>
-  </si>
-  <si>
-    <t>Bagade</t>
-  </si>
-  <si>
     <t>Computer Engineering</t>
   </si>
   <si>
     <t>Assistant Professor</t>
   </si>
   <si>
-    <t>9876543210</t>
-  </si>
-  <si>
-    <t>faculty@college.edu</t>
-  </si>
-  <si>
-    <t>ABCDE1234F</t>
-  </si>
-  <si>
-    <t>Male</t>
-  </si>
-  <si>
-    <t>PhD</t>
-  </si>
-  <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>01-06-2018</t>
-  </si>
-  <si>
-    <t>Permanent</t>
-  </si>
-  <si>
-    <t>CFD</t>
-  </si>
-  <si>
     <t>Rule</t>
   </si>
   <si>
@@ -155,46 +119,190 @@
     <t>Do not delete mandatory columns.</t>
   </si>
   <si>
-    <t>EMP002</t>
-  </si>
-  <si>
-    <t>Preti</t>
-  </si>
-  <si>
     <t>Professor</t>
   </si>
   <si>
-    <t>peeti@gmail.com</t>
-  </si>
-  <si>
-    <t>MMMMM1234F</t>
-  </si>
-  <si>
-    <t>Female</t>
-  </si>
-  <si>
     <t>Mechanical Engineering</t>
   </si>
   <si>
-    <t>EMP004</t>
-  </si>
-  <si>
-    <t>afdsaf</t>
-  </si>
-  <si>
-    <t>dsafs</t>
-  </si>
-  <si>
-    <t>sadfsdf</t>
-  </si>
-  <si>
     <t>Electrical Engineering</t>
   </si>
   <si>
-    <t>asddsa@gmail.com</t>
-  </si>
-  <si>
-    <t>fffff1111S</t>
+    <t>BSCOER001</t>
+  </si>
+  <si>
+    <t>Mech</t>
+  </si>
+  <si>
+    <t>Faculty1</t>
+  </si>
+  <si>
+    <t>111@gmail.com</t>
+  </si>
+  <si>
+    <t>PAN1111111</t>
+  </si>
+  <si>
+    <t>BSCOER002</t>
+  </si>
+  <si>
+    <t>BSCOER003</t>
+  </si>
+  <si>
+    <t>BSCOER004</t>
+  </si>
+  <si>
+    <t>BSCOER005</t>
+  </si>
+  <si>
+    <t>BSCOER006</t>
+  </si>
+  <si>
+    <t>BSCOER007</t>
+  </si>
+  <si>
+    <t>BSCOER008</t>
+  </si>
+  <si>
+    <t>BSCOER009</t>
+  </si>
+  <si>
+    <t>BSCOER010</t>
+  </si>
+  <si>
+    <t>BSCOER011</t>
+  </si>
+  <si>
+    <t>BSCOER012</t>
+  </si>
+  <si>
+    <t>BSCOER013</t>
+  </si>
+  <si>
+    <t>BSCOER014</t>
+  </si>
+  <si>
+    <t>BSCOER015</t>
+  </si>
+  <si>
+    <t>Faculty2</t>
+  </si>
+  <si>
+    <t>Associate Professor</t>
+  </si>
+  <si>
+    <t>222@gmail.com</t>
+  </si>
+  <si>
+    <t>PAN2222222</t>
+  </si>
+  <si>
+    <t>Faculty3</t>
+  </si>
+  <si>
+    <t>PAN3333333</t>
+  </si>
+  <si>
+    <t>PAN4444444</t>
+  </si>
+  <si>
+    <t>PAN5555555</t>
+  </si>
+  <si>
+    <t>PAN6666666</t>
+  </si>
+  <si>
+    <t>PAN7777777</t>
+  </si>
+  <si>
+    <t>PAN8888888</t>
+  </si>
+  <si>
+    <t>PAN9999999</t>
+  </si>
+  <si>
+    <t>PAN11111110</t>
+  </si>
+  <si>
+    <t>PAN12222221</t>
+  </si>
+  <si>
+    <t>PAN13333332</t>
+  </si>
+  <si>
+    <t>Faculty13</t>
+  </si>
+  <si>
+    <t>PAN14444443</t>
+  </si>
+  <si>
+    <t>Faculty14</t>
+  </si>
+  <si>
+    <t>PAN15555554</t>
+  </si>
+  <si>
+    <t>Faculty15</t>
+  </si>
+  <si>
+    <t>PAN16666665</t>
+  </si>
+  <si>
+    <t>Civil</t>
+  </si>
+  <si>
+    <t>Civil Engineering</t>
+  </si>
+  <si>
+    <t>333@gmail.com</t>
+  </si>
+  <si>
+    <t>444@gmail.com</t>
+  </si>
+  <si>
+    <t>555@gmail.com</t>
+  </si>
+  <si>
+    <t>666@gmail.com</t>
+  </si>
+  <si>
+    <t>Elect</t>
+  </si>
+  <si>
+    <t>777@gmail.com</t>
+  </si>
+  <si>
+    <t>888@gmail.com</t>
+  </si>
+  <si>
+    <t>999@gmail.com</t>
+  </si>
+  <si>
+    <t>ENTC</t>
+  </si>
+  <si>
+    <t>e111@gmail.com</t>
+  </si>
+  <si>
+    <t>e222@gmail.com</t>
+  </si>
+  <si>
+    <t>e333@gmail.com</t>
+  </si>
+  <si>
+    <t>Comp</t>
+  </si>
+  <si>
+    <t>c111@gmail.com</t>
+  </si>
+  <si>
+    <t>c222@gmail.com</t>
+  </si>
+  <si>
+    <t>c333@gmail.com</t>
+  </si>
+  <si>
+    <t>ENTC Engineering</t>
   </si>
 </sst>
 </file>
@@ -273,8 +381,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImportTable" displayName="ImportTable" ref="A1:O4">
-  <autoFilter ref="A1:O4"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ImportTable" displayName="ImportTable" ref="A1:O16">
+  <autoFilter ref="A1:O16"/>
   <tableColumns count="15">
     <tableColumn id="1" name="* Employee Code"/>
     <tableColumn id="2" name="* First Name"/>
@@ -581,7 +689,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -649,114 +757,415 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="D2" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="E2" t="s">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="F2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G2" t="s">
-        <v>20</v>
-      </c>
-      <c r="H2" t="s">
-        <v>21</v>
+        <v>34</v>
+      </c>
+      <c r="G2">
+        <v>1111111111</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>40</v>
       </c>
       <c r="I2" t="s">
-        <v>22</v>
-      </c>
-      <c r="J2" t="s">
-        <v>23</v>
-      </c>
-      <c r="K2" t="s">
-        <v>24</v>
-      </c>
-      <c r="L2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N2" t="s">
-        <v>27</v>
-      </c>
-      <c r="O2" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B3" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="D3" t="s">
-        <v>17</v>
+        <v>56</v>
       </c>
       <c r="E3" t="s">
-        <v>52</v>
+        <v>35</v>
       </c>
       <c r="F3" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="G3">
-        <v>7777777777</v>
+        <v>2222222222</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="I3" t="s">
-        <v>50</v>
-      </c>
-      <c r="J3" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4">
+        <v>3333333333</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="I4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B5" t="s">
+        <v>77</v>
+      </c>
+      <c r="D5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E5" t="s">
+        <v>78</v>
+      </c>
+      <c r="F5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G5">
+        <v>4444444444</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="I5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B6" t="s">
+        <v>77</v>
+      </c>
+      <c r="D6" t="s">
+        <v>56</v>
+      </c>
+      <c r="E6" t="s">
+        <v>78</v>
+      </c>
+      <c r="F6" t="s">
+        <v>57</v>
+      </c>
+      <c r="G6">
+        <v>5555555555</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="I6" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" t="s">
+        <v>77</v>
+      </c>
+      <c r="D7" t="s">
+        <v>60</v>
+      </c>
+      <c r="E7" t="s">
+        <v>78</v>
+      </c>
+      <c r="F7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7">
+        <v>6666666666</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="I7" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>47</v>
+      </c>
+      <c r="B8" t="s">
+        <v>83</v>
+      </c>
+      <c r="D8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E8" t="s">
+        <v>36</v>
+      </c>
+      <c r="F8" t="s">
+        <v>34</v>
+      </c>
+      <c r="G8">
+        <v>7777777777</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="I8" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B9" t="s">
+        <v>83</v>
+      </c>
+      <c r="D9" t="s">
+        <v>56</v>
+      </c>
+      <c r="E9" t="s">
+        <v>36</v>
+      </c>
+      <c r="F9" t="s">
+        <v>57</v>
+      </c>
+      <c r="G9">
+        <v>8888888888</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="I9" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>49</v>
+      </c>
+      <c r="B10" t="s">
+        <v>83</v>
+      </c>
+      <c r="D10" t="s">
+        <v>60</v>
+      </c>
+      <c r="E10" t="s">
+        <v>36</v>
+      </c>
+      <c r="F10" t="s">
+        <v>16</v>
+      </c>
+      <c r="G10">
+        <v>9999999999</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="I10" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>50</v>
+      </c>
+      <c r="B11" t="s">
+        <v>87</v>
+      </c>
+      <c r="D11" t="s">
+        <v>39</v>
+      </c>
+      <c r="E11" t="s">
+        <v>95</v>
+      </c>
+      <c r="F11" t="s">
+        <v>34</v>
+      </c>
+      <c r="G11">
+        <v>1111111110</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="I11" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>51</v>
+      </c>
+      <c r="B12" t="s">
+        <v>87</v>
+      </c>
+      <c r="D12" t="s">
+        <v>56</v>
+      </c>
+      <c r="E12" t="s">
+        <v>95</v>
+      </c>
+      <c r="F12" t="s">
+        <v>57</v>
+      </c>
+      <c r="G12">
+        <v>2222222221</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="I12" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>52</v>
+      </c>
+      <c r="B13" t="s">
+        <v>87</v>
+      </c>
+      <c r="D13" t="s">
+        <v>60</v>
+      </c>
+      <c r="E13" t="s">
+        <v>95</v>
+      </c>
+      <c r="F13" t="s">
+        <v>16</v>
+      </c>
+      <c r="G13">
+        <v>3333333332</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="I13" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>53</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B14" t="s">
+        <v>91</v>
+      </c>
+      <c r="D14" t="s">
+        <v>71</v>
+      </c>
+      <c r="E14" t="s">
+        <v>15</v>
+      </c>
+      <c r="F14" t="s">
+        <v>34</v>
+      </c>
+      <c r="G14">
+        <v>4444444443</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="I14" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>54</v>
       </c>
-      <c r="C4" t="s">
+      <c r="B15" t="s">
+        <v>91</v>
+      </c>
+      <c r="D15" t="s">
+        <v>73</v>
+      </c>
+      <c r="E15" t="s">
+        <v>15</v>
+      </c>
+      <c r="F15" t="s">
+        <v>57</v>
+      </c>
+      <c r="G15">
+        <v>5555555554</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="I15" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>55</v>
       </c>
-      <c r="D4" t="s">
-        <v>56</v>
-      </c>
-      <c r="E4" t="s">
-        <v>57</v>
-      </c>
-      <c r="F4" t="s">
-        <v>19</v>
-      </c>
-      <c r="G4">
-        <v>1212121212</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="I4" t="s">
-        <v>59</v>
+      <c r="B16" t="s">
+        <v>91</v>
+      </c>
+      <c r="D16" t="s">
+        <v>75</v>
+      </c>
+      <c r="E16" t="s">
+        <v>15</v>
+      </c>
+      <c r="F16" t="s">
+        <v>16</v>
+      </c>
+      <c r="G16">
+        <v>6666666665</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="I16" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="H3" r:id="rId1"/>
-    <hyperlink ref="H4" r:id="rId2"/>
+    <hyperlink ref="H2" r:id="rId1"/>
+    <hyperlink ref="H3" r:id="rId2"/>
+    <hyperlink ref="H4" r:id="rId3"/>
+    <hyperlink ref="H5" r:id="rId4"/>
+    <hyperlink ref="H8" r:id="rId5"/>
+    <hyperlink ref="H11" r:id="rId6"/>
+    <hyperlink ref="H14" r:id="rId7"/>
+    <hyperlink ref="H6" r:id="rId8"/>
+    <hyperlink ref="H9" r:id="rId9"/>
+    <hyperlink ref="H12" r:id="rId10"/>
+    <hyperlink ref="H15" r:id="rId11"/>
+    <hyperlink ref="H7" r:id="rId12"/>
+    <hyperlink ref="H10" r:id="rId13"/>
+    <hyperlink ref="H13" r:id="rId14"/>
+    <hyperlink ref="H16" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId16"/>
   </tableParts>
 </worksheet>
 </file>
@@ -772,42 +1181,42 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="B2" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B3" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="B4" t="s">
-        <v>36</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="B5" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -815,7 +1224,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -823,31 +1232,31 @@
         <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="B8" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="B9" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="B10" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>